<commit_message>
Improve Zones_Brands.xlsx: styled layout, extra columns, status dropdowns
</commit_message>
<xml_diff>
--- a/Zones_Brands.xlsx
+++ b/Zones_Brands.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -29,10 +29,19 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="12"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <color rgb="00000000"/>
+      <sz val="11"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -41,7 +50,22 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="001F3864"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00305496"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9E1F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
   </fills>
@@ -55,34 +79,42 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00B0B0B0"/>
+        <color rgb="008EA9DB"/>
       </left>
       <right style="thin">
-        <color rgb="00B0B0B0"/>
+        <color rgb="008EA9DB"/>
       </right>
       <top style="thin">
-        <color rgb="00B0B0B0"/>
+        <color rgb="008EA9DB"/>
       </top>
       <bottom style="thin">
-        <color rgb="00B0B0B0"/>
+        <color rgb="008EA9DB"/>
       </bottom>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -448,98 +480,146 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="32" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="7" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="26" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>ZONE:  Central 50</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="22" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
           <t>S.No</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>Brand Name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>GST</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>FSSAI</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="n">
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>GST Number</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>FSSAI Number</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>GST Status</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>FSSAI Status</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Remarks</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1">
+      <c r="A3" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B3" s="4" t="inlineStr">
         <is>
           <t>The Coffee Vault</t>
         </is>
       </c>
-      <c r="C2" s="4" t="inlineStr"/>
-      <c r="D2" s="4" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="n">
+      <c r="C3" s="3" t="inlineStr"/>
+      <c r="D3" s="3" t="inlineStr"/>
+      <c r="E3" s="3" t="inlineStr"/>
+      <c r="F3" s="3" t="inlineStr"/>
+      <c r="G3" s="4" t="inlineStr"/>
+    </row>
+    <row r="4" ht="20" customHeight="1">
+      <c r="A4" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B4" s="6" t="inlineStr">
         <is>
           <t>The Momo Box</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr"/>
-      <c r="D3" s="4" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="n">
+      <c r="C4" s="5" t="inlineStr"/>
+      <c r="D4" s="5" t="inlineStr"/>
+      <c r="E4" s="5" t="inlineStr"/>
+      <c r="F4" s="5" t="inlineStr"/>
+      <c r="G4" s="6" t="inlineStr"/>
+    </row>
+    <row r="5" ht="20" customHeight="1">
+      <c r="A5" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>Umami</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr"/>
-      <c r="D4" s="4" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="n">
+      <c r="C5" s="3" t="inlineStr"/>
+      <c r="D5" s="3" t="inlineStr"/>
+      <c r="E5" s="3" t="inlineStr"/>
+      <c r="F5" s="3" t="inlineStr"/>
+      <c r="G5" s="4" t="inlineStr"/>
+    </row>
+    <row r="6" ht="20" customHeight="1">
+      <c r="A6" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>The Chatpata Affair</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr"/>
-      <c r="D5" s="4" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="n">
+      <c r="C6" s="5" t="inlineStr"/>
+      <c r="D6" s="5" t="inlineStr"/>
+      <c r="E6" s="5" t="inlineStr"/>
+      <c r="F6" s="5" t="inlineStr"/>
+      <c r="G6" s="6" t="inlineStr"/>
+    </row>
+    <row r="7" ht="20" customHeight="1">
+      <c r="A7" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>Sausage Saloon</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr"/>
-      <c r="D6" s="4" t="inlineStr"/>
+      <c r="C7" s="3" t="inlineStr"/>
+      <c r="D7" s="3" t="inlineStr"/>
+      <c r="E7" s="3" t="inlineStr"/>
+      <c r="F7" s="3" t="inlineStr"/>
+      <c r="G7" s="4" t="inlineStr"/>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:G1"/>
+  </mergeCells>
+  <dataValidations count="1">
+    <dataValidation sqref="E3:F7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Choose from the list" prompt="Select status" type="list">
+      <formula1>"Done,Pending,In Process,NA"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -550,170 +630,236 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:G13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="32" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="7" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="26" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>ZONE:  Bennett University</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="22" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
           <t>S.No</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>Brand Name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>GST</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>FSSAI</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="n">
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>GST Number</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>FSSAI Number</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>GST Status</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>FSSAI Status</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Remarks</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1">
+      <c r="A3" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B3" s="4" t="inlineStr">
         <is>
           <t>B2B</t>
         </is>
       </c>
-      <c r="C2" s="4" t="inlineStr"/>
-      <c r="D2" s="4" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="n">
+      <c r="C3" s="3" t="inlineStr"/>
+      <c r="D3" s="3" t="inlineStr"/>
+      <c r="E3" s="3" t="inlineStr"/>
+      <c r="F3" s="3" t="inlineStr"/>
+      <c r="G3" s="4" t="inlineStr"/>
+    </row>
+    <row r="4" ht="20" customHeight="1">
+      <c r="A4" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B4" s="6" t="inlineStr">
         <is>
           <t>Bigg Bear</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr"/>
-      <c r="D3" s="4" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="n">
+      <c r="C4" s="5" t="inlineStr"/>
+      <c r="D4" s="5" t="inlineStr"/>
+      <c r="E4" s="5" t="inlineStr"/>
+      <c r="F4" s="5" t="inlineStr"/>
+      <c r="G4" s="6" t="inlineStr"/>
+    </row>
+    <row r="5" ht="20" customHeight="1">
+      <c r="A5" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>BBF</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr"/>
-      <c r="D4" s="4" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="n">
+      <c r="C5" s="3" t="inlineStr"/>
+      <c r="D5" s="3" t="inlineStr"/>
+      <c r="E5" s="3" t="inlineStr"/>
+      <c r="F5" s="3" t="inlineStr"/>
+      <c r="G5" s="4" t="inlineStr"/>
+    </row>
+    <row r="6" ht="20" customHeight="1">
+      <c r="A6" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>OG Pizza</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr"/>
-      <c r="D5" s="4" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="n">
+      <c r="C6" s="5" t="inlineStr"/>
+      <c r="D6" s="5" t="inlineStr"/>
+      <c r="E6" s="5" t="inlineStr"/>
+      <c r="F6" s="5" t="inlineStr"/>
+      <c r="G6" s="6" t="inlineStr"/>
+    </row>
+    <row r="7" ht="20" customHeight="1">
+      <c r="A7" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>Koby's</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr"/>
-      <c r="D6" s="4" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="n">
+      <c r="C7" s="3" t="inlineStr"/>
+      <c r="D7" s="3" t="inlineStr"/>
+      <c r="E7" s="3" t="inlineStr"/>
+      <c r="F7" s="3" t="inlineStr"/>
+      <c r="G7" s="4" t="inlineStr"/>
+    </row>
+    <row r="8" ht="20" customHeight="1">
+      <c r="A8" s="5" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B8" s="6" t="inlineStr">
         <is>
           <t>The Momo Box</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr"/>
-      <c r="D7" s="4" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="n">
+      <c r="C8" s="5" t="inlineStr"/>
+      <c r="D8" s="5" t="inlineStr"/>
+      <c r="E8" s="5" t="inlineStr"/>
+      <c r="F8" s="5" t="inlineStr"/>
+      <c r="G8" s="6" t="inlineStr"/>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B9" s="4" t="inlineStr">
         <is>
           <t>The Coffee Vault BU</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr"/>
-      <c r="D8" s="4" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="n">
+      <c r="C9" s="3" t="inlineStr"/>
+      <c r="D9" s="3" t="inlineStr"/>
+      <c r="E9" s="3" t="inlineStr"/>
+      <c r="F9" s="3" t="inlineStr"/>
+      <c r="G9" s="4" t="inlineStr"/>
+    </row>
+    <row r="10" ht="20" customHeight="1">
+      <c r="A10" s="5" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B10" s="6" t="inlineStr">
         <is>
           <t>The Chatpata Affair</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr"/>
-      <c r="D9" s="4" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="n">
+      <c r="C10" s="5" t="inlineStr"/>
+      <c r="D10" s="5" t="inlineStr"/>
+      <c r="E10" s="5" t="inlineStr"/>
+      <c r="F10" s="5" t="inlineStr"/>
+      <c r="G10" s="6" t="inlineStr"/>
+    </row>
+    <row r="11" ht="20" customHeight="1">
+      <c r="A11" s="3" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="3" t="inlineStr">
+      <c r="B11" s="4" t="inlineStr">
         <is>
           <t>Eggspert</t>
         </is>
       </c>
-      <c r="C10" s="4" t="inlineStr"/>
-      <c r="D10" s="4" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="n">
+      <c r="C11" s="3" t="inlineStr"/>
+      <c r="D11" s="3" t="inlineStr"/>
+      <c r="E11" s="3" t="inlineStr"/>
+      <c r="F11" s="3" t="inlineStr"/>
+      <c r="G11" s="4" t="inlineStr"/>
+    </row>
+    <row r="12" ht="20" customHeight="1">
+      <c r="A12" s="5" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="3" t="inlineStr">
+      <c r="B12" s="6" t="inlineStr">
         <is>
           <t>Burrito Bros</t>
         </is>
       </c>
-      <c r="C11" s="4" t="inlineStr"/>
-      <c r="D11" s="4" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="n">
+      <c r="C12" s="5" t="inlineStr"/>
+      <c r="D12" s="5" t="inlineStr"/>
+      <c r="E12" s="5" t="inlineStr"/>
+      <c r="F12" s="5" t="inlineStr"/>
+      <c r="G12" s="6" t="inlineStr"/>
+    </row>
+    <row r="13" ht="20" customHeight="1">
+      <c r="A13" s="3" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="3" t="inlineStr">
+      <c r="B13" s="4" t="inlineStr">
         <is>
           <t>Soul Crumb</t>
         </is>
       </c>
-      <c r="C12" s="4" t="inlineStr"/>
-      <c r="D12" s="4" t="inlineStr"/>
+      <c r="C13" s="3" t="inlineStr"/>
+      <c r="D13" s="3" t="inlineStr"/>
+      <c r="E13" s="3" t="inlineStr"/>
+      <c r="F13" s="3" t="inlineStr"/>
+      <c r="G13" s="4" t="inlineStr"/>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:G1"/>
+  </mergeCells>
+  <dataValidations count="1">
+    <dataValidation sqref="E3:F13" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Choose from the list" prompt="Select status" type="list">
+      <formula1>"Done,Pending,In Process,NA"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Combine all zones into single printable sheet with zone section headers
</commit_message>
<xml_diff>
--- a/Zones_Brands.xlsx
+++ b/Zones_Brands.xlsx
@@ -7,10 +7,12 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Central 50" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Bennett University" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Compliance Tracker" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">'Compliance Tracker'!$1:$2</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Compliance Tracker'!$A$1:$H$20</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -18,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -29,7 +31,7 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="14"/>
+      <sz val="16"/>
     </font>
     <font>
       <b val="1"/>
@@ -37,11 +39,16 @@
       <sz val="11"/>
     </font>
     <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="12"/>
+    </font>
+    <font>
       <color rgb="00000000"/>
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -56,6 +63,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00305496"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002E75B6"/>
       </patternFill>
     </fill>
     <fill>
@@ -95,24 +107,28 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -478,24 +494,25 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:H20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
     <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
     <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="28" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1" ht="26" customHeight="1">
+    <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>ZONE:  Central 50</t>
+          <t>BRAND COMPLIANCE TRACKER  (GST / FSSAI)</t>
         </is>
       </c>
     </row>
@@ -507,359 +524,400 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
+          <t>Zone</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
           <t>Brand Name</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>GST Number</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>FSSAI Number</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>GST Status</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>FSSAI Status</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>Remarks</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="20" customHeight="1">
-      <c r="A3" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="B3" s="4" t="inlineStr">
-        <is>
-          <t>The Coffee Vault</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr"/>
-      <c r="D3" s="3" t="inlineStr"/>
-      <c r="E3" s="3" t="inlineStr"/>
-      <c r="F3" s="3" t="inlineStr"/>
-      <c r="G3" s="4" t="inlineStr"/>
+    <row r="3" ht="22" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>▌ Central 50   (5 brands)</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="n"/>
+      <c r="C3" s="4" t="n"/>
+      <c r="D3" s="4" t="n"/>
+      <c r="E3" s="4" t="n"/>
+      <c r="F3" s="4" t="n"/>
+      <c r="G3" s="4" t="n"/>
+      <c r="H3" s="4" t="n"/>
     </row>
     <row r="4" ht="20" customHeight="1">
       <c r="A4" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B4" s="6" t="inlineStr">
         <is>
-          <t>The Momo Box</t>
-        </is>
-      </c>
-      <c r="C4" s="5" t="inlineStr"/>
+          <t>Central 50</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>The Coffee Vault</t>
+        </is>
+      </c>
       <c r="D4" s="5" t="inlineStr"/>
       <c r="E4" s="5" t="inlineStr"/>
       <c r="F4" s="5" t="inlineStr"/>
-      <c r="G4" s="6" t="inlineStr"/>
+      <c r="G4" s="5" t="inlineStr"/>
+      <c r="H4" s="6" t="inlineStr"/>
     </row>
     <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>Umami</t>
-        </is>
-      </c>
-      <c r="C5" s="3" t="inlineStr"/>
-      <c r="D5" s="3" t="inlineStr"/>
-      <c r="E5" s="3" t="inlineStr"/>
-      <c r="F5" s="3" t="inlineStr"/>
-      <c r="G5" s="4" t="inlineStr"/>
+      <c r="A5" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>Central 50</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>The Momo Box</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr"/>
+      <c r="E5" s="7" t="inlineStr"/>
+      <c r="F5" s="7" t="inlineStr"/>
+      <c r="G5" s="7" t="inlineStr"/>
+      <c r="H5" s="8" t="inlineStr"/>
     </row>
     <row r="6" ht="20" customHeight="1">
       <c r="A6" s="5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>The Chatpata Affair</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="inlineStr"/>
+          <t>Central 50</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>Umami</t>
+        </is>
+      </c>
       <c r="D6" s="5" t="inlineStr"/>
       <c r="E6" s="5" t="inlineStr"/>
       <c r="F6" s="5" t="inlineStr"/>
-      <c r="G6" s="6" t="inlineStr"/>
+      <c r="G6" s="5" t="inlineStr"/>
+      <c r="H6" s="6" t="inlineStr"/>
     </row>
     <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="3" t="n">
+      <c r="A7" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>Central 50</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>The Chatpata Affair</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr"/>
+      <c r="E7" s="7" t="inlineStr"/>
+      <c r="F7" s="7" t="inlineStr"/>
+      <c r="G7" s="7" t="inlineStr"/>
+      <c r="H7" s="8" t="inlineStr"/>
+    </row>
+    <row r="8" ht="20" customHeight="1">
+      <c r="A8" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>Central 50</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
         <is>
           <t>Sausage Saloon</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr"/>
-      <c r="D7" s="3" t="inlineStr"/>
-      <c r="E7" s="3" t="inlineStr"/>
-      <c r="F7" s="3" t="inlineStr"/>
-      <c r="G7" s="4" t="inlineStr"/>
+      <c r="D8" s="5" t="inlineStr"/>
+      <c r="E8" s="5" t="inlineStr"/>
+      <c r="F8" s="5" t="inlineStr"/>
+      <c r="G8" s="5" t="inlineStr"/>
+      <c r="H8" s="6" t="inlineStr"/>
+    </row>
+    <row r="9" ht="22" customHeight="1">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>▌ Bennett University   (11 brands)</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="n"/>
+      <c r="C9" s="4" t="n"/>
+      <c r="D9" s="4" t="n"/>
+      <c r="E9" s="4" t="n"/>
+      <c r="F9" s="4" t="n"/>
+      <c r="G9" s="4" t="n"/>
+      <c r="H9" s="4" t="n"/>
+    </row>
+    <row r="10" ht="20" customHeight="1">
+      <c r="A10" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>Bennett University</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>B2B</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr"/>
+      <c r="E10" s="5" t="inlineStr"/>
+      <c r="F10" s="5" t="inlineStr"/>
+      <c r="G10" s="5" t="inlineStr"/>
+      <c r="H10" s="6" t="inlineStr"/>
+    </row>
+    <row r="11" ht="20" customHeight="1">
+      <c r="A11" s="7" t="n">
+        <v>7</v>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>Bennett University</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>Bigg Bear</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr"/>
+      <c r="E11" s="7" t="inlineStr"/>
+      <c r="F11" s="7" t="inlineStr"/>
+      <c r="G11" s="7" t="inlineStr"/>
+      <c r="H11" s="8" t="inlineStr"/>
+    </row>
+    <row r="12" ht="20" customHeight="1">
+      <c r="A12" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>Bennett University</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>BBF</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr"/>
+      <c r="E12" s="5" t="inlineStr"/>
+      <c r="F12" s="5" t="inlineStr"/>
+      <c r="G12" s="5" t="inlineStr"/>
+      <c r="H12" s="6" t="inlineStr"/>
+    </row>
+    <row r="13" ht="20" customHeight="1">
+      <c r="A13" s="7" t="n">
+        <v>9</v>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>Bennett University</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>OG Pizza</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="inlineStr"/>
+      <c r="E13" s="7" t="inlineStr"/>
+      <c r="F13" s="7" t="inlineStr"/>
+      <c r="G13" s="7" t="inlineStr"/>
+      <c r="H13" s="8" t="inlineStr"/>
+    </row>
+    <row r="14" ht="20" customHeight="1">
+      <c r="A14" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>Bennett University</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>Koby's</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr"/>
+      <c r="E14" s="5" t="inlineStr"/>
+      <c r="F14" s="5" t="inlineStr"/>
+      <c r="G14" s="5" t="inlineStr"/>
+      <c r="H14" s="6" t="inlineStr"/>
+    </row>
+    <row r="15" ht="20" customHeight="1">
+      <c r="A15" s="7" t="n">
+        <v>11</v>
+      </c>
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>Bennett University</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>The Momo Box</t>
+        </is>
+      </c>
+      <c r="D15" s="7" t="inlineStr"/>
+      <c r="E15" s="7" t="inlineStr"/>
+      <c r="F15" s="7" t="inlineStr"/>
+      <c r="G15" s="7" t="inlineStr"/>
+      <c r="H15" s="8" t="inlineStr"/>
+    </row>
+    <row r="16" ht="20" customHeight="1">
+      <c r="A16" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>Bennett University</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>The Coffee Vault BU</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr"/>
+      <c r="E16" s="5" t="inlineStr"/>
+      <c r="F16" s="5" t="inlineStr"/>
+      <c r="G16" s="5" t="inlineStr"/>
+      <c r="H16" s="6" t="inlineStr"/>
+    </row>
+    <row r="17" ht="20" customHeight="1">
+      <c r="A17" s="7" t="n">
+        <v>13</v>
+      </c>
+      <c r="B17" s="8" t="inlineStr">
+        <is>
+          <t>Bennett University</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>The Chatpata Affair</t>
+        </is>
+      </c>
+      <c r="D17" s="7" t="inlineStr"/>
+      <c r="E17" s="7" t="inlineStr"/>
+      <c r="F17" s="7" t="inlineStr"/>
+      <c r="G17" s="7" t="inlineStr"/>
+      <c r="H17" s="8" t="inlineStr"/>
+    </row>
+    <row r="18" ht="20" customHeight="1">
+      <c r="A18" s="5" t="n">
+        <v>14</v>
+      </c>
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>Bennett University</t>
+        </is>
+      </c>
+      <c r="C18" s="6" t="inlineStr">
+        <is>
+          <t>Eggspert</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr"/>
+      <c r="E18" s="5" t="inlineStr"/>
+      <c r="F18" s="5" t="inlineStr"/>
+      <c r="G18" s="5" t="inlineStr"/>
+      <c r="H18" s="6" t="inlineStr"/>
+    </row>
+    <row r="19" ht="20" customHeight="1">
+      <c r="A19" s="7" t="n">
+        <v>15</v>
+      </c>
+      <c r="B19" s="8" t="inlineStr">
+        <is>
+          <t>Bennett University</t>
+        </is>
+      </c>
+      <c r="C19" s="8" t="inlineStr">
+        <is>
+          <t>Burrito Bros</t>
+        </is>
+      </c>
+      <c r="D19" s="7" t="inlineStr"/>
+      <c r="E19" s="7" t="inlineStr"/>
+      <c r="F19" s="7" t="inlineStr"/>
+      <c r="G19" s="7" t="inlineStr"/>
+      <c r="H19" s="8" t="inlineStr"/>
+    </row>
+    <row r="20" ht="20" customHeight="1">
+      <c r="A20" s="5" t="n">
+        <v>16</v>
+      </c>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>Bennett University</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>Soul Crumb</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr"/>
+      <c r="E20" s="5" t="inlineStr"/>
+      <c r="F20" s="5" t="inlineStr"/>
+      <c r="G20" s="5" t="inlineStr"/>
+      <c r="H20" s="6" t="inlineStr"/>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:G1"/>
+  <mergeCells count="3">
+    <mergeCell ref="A9:H9"/>
+    <mergeCell ref="A3:H3"/>
+    <mergeCell ref="A1:H1"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="E3:F7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Choose from the list" prompt="Select status" type="list">
+    <dataValidation sqref="F4:G8 F10:G20" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" prompt="Select status" type="list">
       <formula1>"Done,Pending,In Process,NA"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:G13"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="7" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="30" customWidth="1" min="7" max="7"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="26" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>ZONE:  Bennett University</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="22" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>S.No</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Brand Name</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>GST Number</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>FSSAI Number</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>GST Status</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>FSSAI Status</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>Remarks</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="20" customHeight="1">
-      <c r="A3" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="B3" s="4" t="inlineStr">
-        <is>
-          <t>B2B</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr"/>
-      <c r="D3" s="3" t="inlineStr"/>
-      <c r="E3" s="3" t="inlineStr"/>
-      <c r="F3" s="3" t="inlineStr"/>
-      <c r="G3" s="4" t="inlineStr"/>
-    </row>
-    <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="B4" s="6" t="inlineStr">
-        <is>
-          <t>Bigg Bear</t>
-        </is>
-      </c>
-      <c r="C4" s="5" t="inlineStr"/>
-      <c r="D4" s="5" t="inlineStr"/>
-      <c r="E4" s="5" t="inlineStr"/>
-      <c r="F4" s="5" t="inlineStr"/>
-      <c r="G4" s="6" t="inlineStr"/>
-    </row>
-    <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>BBF</t>
-        </is>
-      </c>
-      <c r="C5" s="3" t="inlineStr"/>
-      <c r="D5" s="3" t="inlineStr"/>
-      <c r="E5" s="3" t="inlineStr"/>
-      <c r="F5" s="3" t="inlineStr"/>
-      <c r="G5" s="4" t="inlineStr"/>
-    </row>
-    <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="B6" s="6" t="inlineStr">
-        <is>
-          <t>OG Pizza</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="inlineStr"/>
-      <c r="D6" s="5" t="inlineStr"/>
-      <c r="E6" s="5" t="inlineStr"/>
-      <c r="F6" s="5" t="inlineStr"/>
-      <c r="G6" s="6" t="inlineStr"/>
-    </row>
-    <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>Koby's</t>
-        </is>
-      </c>
-      <c r="C7" s="3" t="inlineStr"/>
-      <c r="D7" s="3" t="inlineStr"/>
-      <c r="E7" s="3" t="inlineStr"/>
-      <c r="F7" s="3" t="inlineStr"/>
-      <c r="G7" s="4" t="inlineStr"/>
-    </row>
-    <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="B8" s="6" t="inlineStr">
-        <is>
-          <t>The Momo Box</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="inlineStr"/>
-      <c r="D8" s="5" t="inlineStr"/>
-      <c r="E8" s="5" t="inlineStr"/>
-      <c r="F8" s="5" t="inlineStr"/>
-      <c r="G8" s="6" t="inlineStr"/>
-    </row>
-    <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="3" t="n">
-        <v>7</v>
-      </c>
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>The Coffee Vault BU</t>
-        </is>
-      </c>
-      <c r="C9" s="3" t="inlineStr"/>
-      <c r="D9" s="3" t="inlineStr"/>
-      <c r="E9" s="3" t="inlineStr"/>
-      <c r="F9" s="3" t="inlineStr"/>
-      <c r="G9" s="4" t="inlineStr"/>
-    </row>
-    <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="5" t="n">
-        <v>8</v>
-      </c>
-      <c r="B10" s="6" t="inlineStr">
-        <is>
-          <t>The Chatpata Affair</t>
-        </is>
-      </c>
-      <c r="C10" s="5" t="inlineStr"/>
-      <c r="D10" s="5" t="inlineStr"/>
-      <c r="E10" s="5" t="inlineStr"/>
-      <c r="F10" s="5" t="inlineStr"/>
-      <c r="G10" s="6" t="inlineStr"/>
-    </row>
-    <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="3" t="n">
-        <v>9</v>
-      </c>
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>Eggspert</t>
-        </is>
-      </c>
-      <c r="C11" s="3" t="inlineStr"/>
-      <c r="D11" s="3" t="inlineStr"/>
-      <c r="E11" s="3" t="inlineStr"/>
-      <c r="F11" s="3" t="inlineStr"/>
-      <c r="G11" s="4" t="inlineStr"/>
-    </row>
-    <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="5" t="n">
-        <v>10</v>
-      </c>
-      <c r="B12" s="6" t="inlineStr">
-        <is>
-          <t>Burrito Bros</t>
-        </is>
-      </c>
-      <c r="C12" s="5" t="inlineStr"/>
-      <c r="D12" s="5" t="inlineStr"/>
-      <c r="E12" s="5" t="inlineStr"/>
-      <c r="F12" s="5" t="inlineStr"/>
-      <c r="G12" s="6" t="inlineStr"/>
-    </row>
-    <row r="13" ht="20" customHeight="1">
-      <c r="A13" s="3" t="n">
-        <v>11</v>
-      </c>
-      <c r="B13" s="4" t="inlineStr">
-        <is>
-          <t>Soul Crumb</t>
-        </is>
-      </c>
-      <c r="C13" s="3" t="inlineStr"/>
-      <c r="D13" s="3" t="inlineStr"/>
-      <c r="E13" s="3" t="inlineStr"/>
-      <c r="F13" s="3" t="inlineStr"/>
-      <c r="G13" s="4" t="inlineStr"/>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:G1"/>
-  </mergeCells>
-  <dataValidations count="1">
-    <dataValidation sqref="E3:F13" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Choose from the list" prompt="Select status" type="list">
-      <formula1>"Done,Pending,In Process,NA"</formula1>
-    </dataValidation>
-  </dataValidations>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
</xml_diff>